<commit_message>
relecture finale + biblio
</commit_message>
<xml_diff>
--- a/Papier/ToSend/VerstraeteGuenette_References.xlsx
+++ b/Papier/ToSend/VerstraeteGuenette_References.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t xml:space="preserve">Part number</t>
   </si>
@@ -31,7 +31,37 @@
     <t xml:space="preserve">DOI_Reference</t>
   </si>
   <si>
-    <t xml:space="preserve">Aubreton, Robert. 1980. Anthologie grecque. Tome XIII: Anthologie de Planude. Vol. XIII. XIII vols. Paris: Les Belles Lettres.</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Aubreton, Robert. 1980. </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Anthologie grecque. Tome XIII: Anthologie de Planude. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Paris: Les Belles Lettres.</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Benkler, Yochai, Aaron Shaw, and Benjamin Mako Hill. 2015. “Peer Production: A Form of Collective Intelligence.” In Handbook of Collective Intelligence, edited by Thomas Malone and Michael Bernstein, 175–204. Cambridge, Massachusetts: MIT Press.</t>
@@ -76,7 +106,37 @@
     <t xml:space="preserve">Gow, Andrew Sydenham Farrar, and Denys Lionel Page. 1965. The Greek anthology. Hellenistic epigrams. Vol. 2. Cambridge: Cambridge University Press.</t>
   </si>
   <si>
-    <t xml:space="preserve">Irigoin, Jean, and Francesca Maltomini. 2017. Anthologie grecque. Tome IX: Anthologie palatine, Livre X. Translated by Pierre Laurens. 2nd ed. Vol. IX. XIII vols. Paris: Les Belles Lettres.</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Irigoin, Jean, and Francesca Maltomini. 2017. </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Anthologie grecque. Tome IX: Anthologie palatine, Livre X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. Paris: Les Belles Lettres.</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Lévy, Pierre. 1994. L’intelligence collective : pour une anthropologie du cyberspace. Paris: La Découverte.</t>
@@ -97,7 +157,7 @@
     <t xml:space="preserve">10.1145/3306446.3340822.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sahle, Patrick. 2017. “2. What Is a Scholarly Digital Edition?” In Digital Scholarly Editing : Theories and Practices, edited by Matthew James Driscoll and Elena Pierazzo, 19–39. Digital Humanities Series. Cambridge: Open Book Publishers.</t>
+    <t xml:space="preserve">Sahle, Patrick. 2016. “2. What Is a Scholarly Digital Edition?” In Digital Scholarly Editing: Theories and Practices, edited by Matthew James Driscoll and Elena Pierazzo, 19–39. Digital Humanities Series. Cambridge: Open Book Publishers.</t>
   </si>
   <si>
     <t xml:space="preserve">Santos, Veronica, Daniel Schwabe, and Sérgio Lifschitz. 2024. “Can You Trust Wikidata?” Semantic Web 15 (6): 2271–92. </t>
@@ -112,7 +172,7 @@
     <t xml:space="preserve">10.3917/ina.sever.2021.01</t>
   </si>
   <si>
-    <t xml:space="preserve">Shenoy, Kartik, Filip Ilievski, Daniel Garijo, Daniel Schwabe, and Pedro Szekely. 2022. “A Study of the Quality of Wikidata.” Journal of Web Semantics 72:100679.</t>
+    <t xml:space="preserve">Shenoy, Kartik, Filip Ilievski, Daniel Garijo, Daniel Schwabe, and Pedro Szekely. 2022. “A Study of the Quality of Wikidata.” Journal of Web Semantics 72 (100679).</t>
   </si>
   <si>
     <t xml:space="preserve">10.1016/j.websem.2021.100679</t>
@@ -121,52 +181,199 @@
     <t xml:space="preserve">Surowiecki, James. 2004. The Wisdom of Crowds: Why the Many Are Smarter than the Few and How Collective Wisdom Shapes Business, Economies, Societies, and Nations. New York: Doubleday.</t>
   </si>
   <si>
+    <t xml:space="preserve">Thornton, Katherine, Harold Solbrig, Gregory S. Stupp, Jose Emilio Labra Gayo, Daniel Mietchen, Eric Prud’hommeaux, and Andra Waagmeester. 2019. “Using Shape Expressions (ShEx) to Share RDF Data Models and to Guide Curation with Rigorous Validation.” In The Semantic Web, edited by Pascal Hitzler, Miriam Fernández, Krzysztof Janowicz, Amrapali Zaveri, Alasdair J.G. Gray, Vanessa Lopez, Armin Haller, and Karl Hammar, 11503:606–20. Lecture Notes in Computer Science. Cham: Springer International Publishing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1007/978-3-030-21348-0_39</t>
+  </si>
+  <si>
     <t xml:space="preserve">Thornton, Katherine, Kenneth Seals Nutt, and Anne Chen. 2024. “Encoding Archaeological Data Models as Wikidata Schemas: Utilizing Shape Expressions to Structure Collaborative Linked Open Data for Digital Storytelling Within the International Dura-Europos Archive.” The International Journal of Technology, Knowledge, and Society 21 (1): 69–83. </t>
   </si>
   <si>
     <t xml:space="preserve">10.18848/1832-3669/CGP/v21i01/69-83</t>
   </si>
   <si>
-    <t xml:space="preserve">Thornton, Katherine, Harold Solbrig, Gregory S. Stupp, Jose Emilio Labra Gayo, Daniel Mietchen, Eric Prud’hommeaux, and Andra Waagmeester. 2019. “Using Shape Expressions (ShEx) to Share RDF Data Models and to Guide Curation with Rigorous Validation.” In The Semantic Web, edited by Pascal Hitzler, Miriam Fernández, Krzysztof Janowicz, Amrapali Zaveri, Alasdair J.G. Gray, Vanessa Lopez, Armin Haller, and Karl Hammar, 11503:606–20. Lecture Notes in Computer Science. Cham: Springer International Publishing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.1007/978-3-030-21348-0_39</t>
-  </si>
-  <si>
     <t xml:space="preserve">Van Veen, Theo. 2019. “Wikidata: From ‘an’ Identifier to ‘the’ Identifier.” Information Technology and Libraries 38 (2): 72–81.</t>
   </si>
   <si>
     <t xml:space="preserve">10.6017/ital.v38i2.10886</t>
   </si>
   <si>
-    <t xml:space="preserve">Verstraete, Mathilde. 2024. “Dynamiques auctoriales au sein du projet d’édition numérique collaborative de l’Anthologie grecque.” Sens Public. http://sens-public.org/articles/1692/.</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Verstraete, Mathilde. 2024. “Dynamiques auctoriales au sein du projet d’édition numérique collaborative de l’</t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Anthologie grecque</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.” Sens Public. http://sens-public.org/articles/1692/.</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Verstraete, Mathilde, and Margot Mellet. 2024. “Passés et présents anthologiques. Le projet d’édition numérique collaborative de l’Anthologie grecque.” In Communautés et pratiques d’écritures des patrimoines et des mémoires, edited by Nicolas Sauret and Marta Severo, 67–80. Paris: Presses universitaires de Paris-Nanterre.</t>
   </si>
   <si>
+    <t xml:space="preserve">Vitali-Rosati, Marcello, Servanne Monjour, Joana Casenave, Elsa Bouchard, and Margot Mellet. 2020. “Editorializing the Greek Anthology: The Palatin Manuscript as a Collective Imaginary.” Digital Humanities Quarterly 14 (1).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vitali-Rosati, Marcello, Margot Mellet, Servanne Monjour, Antoine Fauchié, Timothée Guicherd, David Larlet, and Enrico Agostini-Marchese. 2021. “L’épopée numérique de l’Anthologie grecque : entre questions épistémologiques, modèles techniques et dynamiques collaboratives.” Sens public. </t>
   </si>
   <si>
     <t xml:space="preserve">10.7202/1089649ar</t>
   </si>
   <si>
-    <t xml:space="preserve">Vitali-Rosati, Marcello, Servanne Monjour, Joana Casenave, Elsa Bouchard, and Margot Mellet. 2020. “Editorializing the Greek Anthology: The Palatin Manuscript as a Collective Imaginary.” Digital Humanities Quarterly 14 (1).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waltz, Pierre. 1931. Anthologie grecque. Tome III : Anthologie palatine, Livre VI. XIII vols. Paris: Les Belles Lettres.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waltz, Pierre. 1960. Anthologie grecque. Tome V : Anthologie palatine, Livre VII, Épigrammes 364-748. Translated by Edouard Des Places, M. Dumitrescu, H. Le Maitre, and G. Soury. Paris: Les Belles Lettres.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waltz, Pierre. 1974. Anthologie Grecque. Tome VIII: Anthologie Palatine, Livre IX, Épigrammes 359-827. Edited by Jean Irigoin, Pierre Laurens, and G. Soury. Paris: Les Belles Lettres.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waltz, Pierre. 2003. Anthologie Grecque. Tome II : Anthologie Palatine, Livre V. Edited by Jean Irigoin. Paris: Les Belles Lettres.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waltz, Pierre, Jean Guillon, Jean Irigoin, P. Camelot, Alphonse Dain, Edouard Des Places, A.-M. Desrousseaux, et al. 1929. “Anthologie Grecque.” Paris: Les Belles Lettres.</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Waltz, Pierre. 1931. </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Anthologie grecque. Tome III: Anthologie palatine, Livre VI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. Paris: Les Belles Lettres.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Waltz, Pierre. 1960. </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Anthologie grecque. Tome V: Anthologie palatine, Livre VII, Épigrammes 364-748</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. Paris: Les Belles Lettres.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Waltz, Pierre. 1974. </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Anthologie Grecque. Tome VIII: Anthologie Palatine, Livre IX, Épigrammes 359-827</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. Paris: Les Belles Lettres.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Waltz, Pierre. 2003. </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Anthologie Grecque. Tome II: Anthologie Palatine, Livre V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. Paris: Les Belles Lettres.</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Zhao, Fudie. 2023. “A Systematic Review of Wikidata in Digital Humanities Projects.” Digital Scholarship in the Humanities 38 (2): 852–74. </t>
@@ -182,7 +389,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -207,6 +414,14 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -478,7 +693,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C1048576"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.52"/>
@@ -504,7 +719,7 @@
       </c>
       <c r="C2" s="5"/>
     </row>
-    <row r="3" customFormat="false" ht="55.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3"/>
       <c r="B3" s="6" t="s">
         <v>4</v>
@@ -529,7 +744,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="s">
         <v>9</v>
@@ -538,7 +753,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3"/>
       <c r="B7" s="6" t="s">
         <v>11</v>
@@ -547,7 +762,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3"/>
       <c r="B8" s="6" t="s">
         <v>13</v>
@@ -572,7 +787,7 @@
       </c>
       <c r="C10" s="4"/>
     </row>
-    <row r="11" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="28.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="s">
         <v>18</v>
       </c>
@@ -595,7 +810,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
         <v>23</v>
       </c>
@@ -603,12 +818,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
         <v>26</v>
       </c>
@@ -624,7 +839,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
         <v>30</v>
       </c>
@@ -637,7 +852,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="109.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="s">
         <v>33</v>
       </c>
@@ -645,7 +860,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
         <v>35</v>
       </c>
@@ -653,7 +868,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
         <v>37</v>
       </c>
@@ -661,7 +876,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="42.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="s">
         <v>39</v>
       </c>
@@ -671,16 +886,16 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C26" s="7" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="6" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>43</v>
       </c>
     </row>
@@ -689,17 +904,17 @@
         <v>44</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="28.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="28.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="6" t="s">
         <v>47</v>
       </c>
@@ -708,15 +923,12 @@
       <c r="B32" s="6" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="6" t="s">
+      <c r="C32" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="7" t="s">
-        <v>50</v>
-      </c>
-    </row>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>